<commit_message>
docs(scrum): rebalancear asignacion modular entre integrantes y actualizar entregables
</commit_message>
<xml_diff>
--- a/DOCUMENTACIÓN/BITACORA_DAILY_SCRUM.xlsx
+++ b/DOCUMENTACIÓN/BITACORA_DAILY_SCRUM.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="179">
   <si>
     <t>BITÁCORA DAILY SCRUM — SEGUIMIENTO DE EQUIPO (SPRINT 2)</t>
   </si>
   <si>
-    <t>Integrante: Miguel  |  Módulos Asignados: Tickets, Incidentes, Solicitudes, Seguridad, Plataforma, Operación, Reportes</t>
+    <t>Integrante: Miguel  |  Módulos Asignados: Tickets, Incidentes, Solicitudes, Reportes, Plataforma, Operación</t>
   </si>
   <si>
     <t/>
@@ -182,13 +182,13 @@
     <t>Ninguno. Build exitoso (Code 0) y listo para revisión con el docente.</t>
   </si>
   <si>
-    <t>Integrante: Lourdes  |  Módulos Asignados: Catálogo de Servicios y Acuerdos de Nivel de Servicio (SLA)</t>
+    <t>Integrante: Lourdes  |  Módulos Asignados: Catálogo de Servicios, Acuerdos SLA y Gestión de Activos TI (HAM/SAM)</t>
   </si>
   <si>
     <t>HU-17 (Gestión de Acuerdos de Nivel de Servicio - SLA)</t>
   </si>
   <si>
-    <t>Planificación de compromisos del Sprint 2 enfocados en la gobernanza de SLA y formularios de servicio.</t>
+    <t>Planificación de compromisos del Sprint 2 enfocados en la gobernanza de SLA y gestión de activos.</t>
   </si>
   <si>
     <t>Revisar la estructura de Acuerdos SLA (P1 a P4) y especificación de tiempos de primera respuesta y resolución.</t>
@@ -224,58 +224,55 @@
     <t>HU-17 / HU-18</t>
   </si>
   <si>
-    <t>Finalicé y verifiqué los 3 escenarios de aceptación de HU-17.</t>
-  </si>
-  <si>
-    <t>Iniciar HU-18 analizando el diseñador de campos dinámicos para servicios individuales en src/modules/servicios.</t>
+    <t>Finalicé y verifiqué los 3 escenarios de aceptación de HU-17 (SLA).</t>
+  </si>
+  <si>
+    <t>Iniciar HU-18 analizando el inventario maestro de activos y el módulo de control de licencias SAM.</t>
   </si>
   <si>
     <t>Ninguno. HU-17 completada satisfactoriamente.</t>
   </si>
   <si>
-    <t>HU-18 (Diseñador Dinámico de Campos de Servicios)</t>
-  </si>
-  <si>
-    <t>Analicé los tipos de campos requeridos (texto, número, fecha, selector) por servicio.</t>
-  </si>
-  <si>
-    <t>Desarrollar los componentes UI del diseñador de campos en src/modules/servicios/admin/servicios/[id]/formulario.</t>
-  </si>
-  <si>
-    <t>Desarrollé los controles de entrada y la lista de campos configurables.</t>
-  </si>
-  <si>
-    <t>Implementar el panel de previsualización interactiva del formulario del servicio en tiempo real.</t>
-  </si>
-  <si>
-    <t>Implementé el panel de previsualización en vivo del formulario generado.</t>
-  </si>
-  <si>
-    <t>Conectar el guardado de esquemas dinámicos en base de datos con el controlador del servicio.</t>
-  </si>
-  <si>
-    <t>Sincronización del estado de formulario al alternar entre servicios; se corrigió con key reactiva.</t>
-  </si>
-  <si>
-    <t>Conecté la persistencia de esquemas dinámicos por servicio.</t>
-  </si>
-  <si>
-    <t>Implementar las validaciones reactivas con esquemas Zod dinámicos generados al vuelo.</t>
-  </si>
-  <si>
-    <t>Implementé la validación de campos obligatorios en el catálogo del solicitante.</t>
-  </si>
-  <si>
-    <t>Realizar pruebas completas de diseño, renderizado y guardado de solicitudes con campos dinámicos.</t>
-  </si>
-  <si>
-    <t>Comprobé que los formularios dinámicos se renderizan y validan sin fallas.</t>
-  </si>
-  <si>
-    <t>Validación de tipado estricto en src/modules/servicios, verificación de compilación y cierre de Sprint.</t>
-  </si>
-  <si>
-    <t>Ninguno. Todas las historias asignadas quedaron en columna Hecho.</t>
+    <t>HU-18 (Inventario de Activos TI y Control SAM de Licencias)</t>
+  </si>
+  <si>
+    <t>Analicé el modelo de datos de activos de hardware, software y asignación de custodios.</t>
+  </si>
+  <si>
+    <t>Desarrollar la pantalla de alta de activo con número de serie y custodia en src/modules/activos.</t>
+  </si>
+  <si>
+    <t>Desarrollé el formulario de registro de activos con validación de unicidad de serie.</t>
+  </si>
+  <si>
+    <t>Implementar el control de licenciamiento SAM calculando licencias compradas vs asignadas.</t>
+  </si>
+  <si>
+    <t>Implementé el cálculo automático del porcentaje de ocupación de licencias.</t>
+  </si>
+  <si>
+    <t>Diseñar el semáforo visual de cumplimiento SAM (verde &lt;80%, ámbar 80-99%, rojo 100%+).</t>
+  </si>
+  <si>
+    <t>Diseñé los indicadores del semáforo SAM en la vista de gestión de activos.</t>
+  </si>
+  <si>
+    <t>Implementar el bloqueo que impide asignar licencias cuando se sobrepasa el cupo contratado.</t>
+  </si>
+  <si>
+    <t>Implementé el bloqueo preventivo contra sobreasignación de licencias en activos.</t>
+  </si>
+  <si>
+    <t>Pruebas integrales de registro patrimonial, asignación a colaboradores y semáforo de licencias.</t>
+  </si>
+  <si>
+    <t>Comprobé la consistencia del inventario de activos y el cumplimiento SAM.</t>
+  </si>
+  <si>
+    <t>Revisión final de código en src/modules/servicios y src/modules/activos, prueba de build y cierre de Sprint.</t>
+  </si>
+  <si>
+    <t>Ninguno. Ambas historias finalizadas y listas para la presentación académica.</t>
   </si>
   <si>
     <t>Integrante: Alexis  |  Módulos Asignados: Gestión de Problemas y Gestión del Conocimiento</t>
@@ -371,7 +368,7 @@
     <t>Ninguno. Ambas historias operativas al 100%.</t>
   </si>
   <si>
-    <t>Integrante: Junior  |  Módulos Asignados: Identidades, Organización y Gestión de Proveedores</t>
+    <t>Integrante: Junior  |  Módulos Asignados: Seguridad de Acceso, Identidades (IAM), Organización y Proveedores</t>
   </si>
   <si>
     <t>HU-21 (Departamentos TI y Grupos Resolutores N1/N2/N3)</t>
@@ -458,19 +455,19 @@
     <t>Comprobé el funcionamiento exacto de los turnos y ausencias en la mesa de soporte.</t>
   </si>
   <si>
-    <t>Revisión final de contratos en src/modules/organizacion, verificación de compilación y cierre de Sprint.</t>
+    <t>Revisión final de contratos en src/modules/organizacion y src/modules/seguridad, verificación de compilación y cierre de Sprint.</t>
   </si>
   <si>
     <t>Ninguno. HU-21 y HU-22 en estado Hecho.</t>
   </si>
   <si>
-    <t>Integrante: Nain  |  Módulos Asignados: Gestión de Cambios, Gestión de Activos TI (HAM/SAM) y CMDB</t>
+    <t>Integrante: Nain  |  Módulos Asignados: Gestión de Cambios (Change Enablement) y CMDB (SACM)</t>
   </si>
   <si>
     <t>HU-23 (Solicitud de Cambio - RFC y Ventanas de Mantenimiento)</t>
   </si>
   <si>
-    <t>Planificación de compromisos del Sprint 2 enfocados en Change Enablement y gestión de activos.</t>
+    <t>Planificación de compromisos del Sprint 2 enfocados en Change Enablement y configuración CMDB.</t>
   </si>
   <si>
     <t>Revisar la estructura del formulario de RFC y los requerimientos de plan de rollback en ITIL 4.</t>
@@ -509,52 +506,52 @@
     <t>Completé y verifiqué los escenarios de aceptación de HU-23.</t>
   </si>
   <si>
-    <t>Iniciar HU-24 analizando el inventario maestro de activos y el módulo de gestión de licencias SAM.</t>
+    <t>Iniciar HU-24 analizando el módulo de configuración CMDB, registro de CIs y relaciones de infraestructura.</t>
   </si>
   <si>
     <t>Ninguno. HU-23 concluida exitosamente.</t>
   </si>
   <si>
-    <t>HU-24 (Inventario de Activos TI y Control SAM de Licencias)</t>
-  </si>
-  <si>
-    <t>Analicé el modelo de datos de activos de hardware, software y asignación de custodios.</t>
-  </si>
-  <si>
-    <t>Desarrollar la pantalla de alta de activo con número de serie y custodia en src/modules/activos.</t>
-  </si>
-  <si>
-    <t>Desarrollé el formulario de registro de activos con validación de unicidad de serie.</t>
-  </si>
-  <si>
-    <t>Implementar el control de licenciamiento SAM calculando licencias compradas vs asignadas.</t>
-  </si>
-  <si>
-    <t>Implementé el cálculo automático del porcentaje de ocupación de licencias.</t>
-  </si>
-  <si>
-    <t>Diseñar el semáforo visual de cumplimiento SAM (verde &lt;80%, ámbar 80-99%, rojo 100%+).</t>
-  </si>
-  <si>
-    <t>Diseñé los indicadores del semáforo SAM en la vista de gestión de activos.</t>
-  </si>
-  <si>
-    <t>Implementar el bloqueo que impide asignar licencias cuando se sobrepasa el cupo contratado.</t>
-  </si>
-  <si>
-    <t>Implementé el bloqueo preventivo contra sobreasignación de licencias en activos.</t>
-  </si>
-  <si>
-    <t>Pruebas integrales de registro patrimonial, asignación a colaboradores y semáforo de licencias.</t>
-  </si>
-  <si>
-    <t>Comprobé la consistencia del inventario de activos y el cumplimiento SAM.</t>
-  </si>
-  <si>
-    <t>Revisión final de código en src/modules/cambios y src/modules/activos, prueba de build y cierre de Sprint.</t>
-  </si>
-  <si>
-    <t>Ninguno. Ambas historias finalizadas y listas para la presentación académica.</t>
+    <t>HU-24 (Elementos de Configuración CIs y Líneas Base en CMDB)</t>
+  </si>
+  <si>
+    <t>Analicé el esquema de clases de CI (servidores, redes, bases de datos) y relaciones en src/modules/cmdb.</t>
+  </si>
+  <si>
+    <t>Desarrollar la pantalla de registro y tipificación de Elementos de Configuración en la CMDB.</t>
+  </si>
+  <si>
+    <t>Desarrollé la vista de alta y edición de CIs con campos de versión y criticidad.</t>
+  </si>
+  <si>
+    <t>Implementar el gestor de relaciones padre-hijo (Depende de, Conectado a, Aloja a) entre componentes.</t>
+  </si>
+  <si>
+    <t>Implementé la persistencia de relaciones lógicas y físicas en la tabla de relaciones CMDB.</t>
+  </si>
+  <si>
+    <t>Construir el validador de integridad para prevenir relaciones circulares en el grafo de infraestructura.</t>
+  </si>
+  <si>
+    <t>Evitar bucles infinitos en árboles de dependencia profundos; se resolvió con detección de ciclos DFS.</t>
+  </si>
+  <si>
+    <t>Implementé el algoritmo de prevención de ciclos en el grafo de CIs.</t>
+  </si>
+  <si>
+    <t>Desarrollar la funcionalidad de auditoría de líneas base y detección de discrepancias no autorizadas.</t>
+  </si>
+  <si>
+    <t>Implementé el reporte de auditoría de líneas base de configuración.</t>
+  </si>
+  <si>
+    <t>Pruebas integrales de vinculación entre Solicitudes de Cambio (RFC) y CIs afectados en la CMDB.</t>
+  </si>
+  <si>
+    <t>Comprobé que los cambios reflejan con exactitud el impacto sobre los CIs de la CMDB.</t>
+  </si>
+  <si>
+    <t>Revisión final de código en src/modules/cambios y src/modules/cmdb, prueba de compilación y cierre de Sprint.</t>
   </si>
 </sst>
 </file>
@@ -1502,7 +1499,7 @@
         <v>78</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>79</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1513,10 +1510,10 @@
         <v>72</v>
       </c>
       <c r="C14" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>81</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>20</v>
@@ -1530,10 +1527,10 @@
         <v>68</v>
       </c>
       <c r="C15" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>82</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>83</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>20</v>
@@ -1547,13 +1544,13 @@
         <v>68</v>
       </c>
       <c r="C16" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>85</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1589,7 +1586,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1627,13 +1624,13 @@
         <v>8</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>89</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>90</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>20</v>
@@ -1644,13 +1641,13 @@
         <v>13</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>91</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>92</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>20</v>
@@ -1661,13 +1658,13 @@
         <v>17</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>94</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>20</v>
@@ -1678,13 +1675,13 @@
         <v>21</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>95</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>96</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>20</v>
@@ -1695,13 +1692,13 @@
         <v>25</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>97</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>20</v>
@@ -1712,16 +1709,16 @@
         <v>28</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="7" t="s">
         <v>101</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1729,13 +1726,13 @@
         <v>33</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>105</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>20</v>
@@ -1746,16 +1743,16 @@
         <v>37</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="E12" s="7" t="s">
         <v>107</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1763,13 +1760,13 @@
         <v>41</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>110</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>20</v>
@@ -1780,13 +1777,13 @@
         <v>44</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C14" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>111</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>112</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>20</v>
@@ -1797,13 +1794,13 @@
         <v>47</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C15" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>114</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>20</v>
@@ -1814,16 +1811,16 @@
         <v>51</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C16" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>116</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -1859,7 +1856,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1897,13 +1894,13 @@
         <v>8</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>120</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>121</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>20</v>
@@ -1914,13 +1911,13 @@
         <v>13</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>122</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>123</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>20</v>
@@ -1931,13 +1928,13 @@
         <v>17</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>124</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>125</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>20</v>
@@ -1948,13 +1945,13 @@
         <v>21</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>126</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>127</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>20</v>
@@ -1965,13 +1962,13 @@
         <v>25</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>128</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>129</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>20</v>
@@ -1982,16 +1979,16 @@
         <v>28</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="7" t="s">
         <v>132</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1999,13 +1996,13 @@
         <v>33</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>135</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>136</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>20</v>
@@ -2016,13 +2013,13 @@
         <v>37</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>137</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>138</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>20</v>
@@ -2033,16 +2030,16 @@
         <v>41</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>140</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2050,13 +2047,13 @@
         <v>44</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C14" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>142</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>143</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>20</v>
@@ -2067,13 +2064,13 @@
         <v>47</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C15" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>145</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>20</v>
@@ -2084,16 +2081,16 @@
         <v>51</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C16" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>147</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -2129,7 +2126,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2167,13 +2164,13 @@
         <v>8</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>152</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>20</v>
@@ -2184,13 +2181,13 @@
         <v>13</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>153</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>154</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>20</v>
@@ -2201,13 +2198,13 @@
         <v>17</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>155</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>156</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>20</v>
@@ -2218,16 +2215,16 @@
         <v>21</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>158</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2235,13 +2232,13 @@
         <v>25</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>160</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>161</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>20</v>
@@ -2252,16 +2249,16 @@
         <v>28</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="7" t="s">
         <v>164</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2269,13 +2266,13 @@
         <v>33</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>167</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>168</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>20</v>
@@ -2286,13 +2283,13 @@
         <v>37</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>169</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>170</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>20</v>
@@ -2303,16 +2300,16 @@
         <v>41</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>172</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2320,7 +2317,7 @@
         <v>44</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>173</v>
@@ -2337,7 +2334,7 @@
         <v>47</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>175</v>
@@ -2354,7 +2351,7 @@
         <v>51</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>177</v>
@@ -2363,7 +2360,7 @@
         <v>178</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>179</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(scrum): clarificar referencia de Alexis (Darhien) en asignacion y scrum
</commit_message>
<xml_diff>
--- a/DOCUMENTACIÓN/BITACORA_DAILY_SCRUM.xlsx
+++ b/DOCUMENTACIÓN/BITACORA_DAILY_SCRUM.xlsx
@@ -3,6 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9000" activeTab="2"/>
+  </bookViews>
   <sheets>
     <sheet sheetId="1" name="Miguel" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Lourdes" state="visible" r:id="rId5"/>
@@ -275,7 +278,7 @@
     <t>Ninguno. Ambas historias finalizadas y listas para la presentación académica.</t>
   </si>
   <si>
-    <t>Integrante: Alexis  |  Módulos Asignados: Gestión de Problemas y Gestión del Conocimiento</t>
+    <t>Integrante: Alexis (Darhien)  |  Módulos Asignados: Gestión de Problemas y Gestión del Conocimiento</t>
   </si>
   <si>
     <t>HU-19 (Registro de Problemas y Análisis Causa Raíz - RCA)</t>
@@ -568,23 +571,27 @@
     </font>
     <font>
       <b/>
+      <charset val="134"/>
       <color rgb="FFFFFFFF"/>
       <sz val="14"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <charset val="134"/>
       <color rgb="FF2D3748"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <charset val="134"/>
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
+      <charset val="134"/>
       <sz val="9"/>
       <name val="Arial"/>
     </font>
@@ -598,27 +605,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A365D"/>
+        <fgColor theme="3" tint="-0.25"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2E8F0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2B6CB0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF7FAFC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A365D"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -664,7 +676,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -672,8 +684,14 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -681,11 +699,8 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1020,14 +1035,13 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="4" x14ac:dyDescent="0" defaultColWidth="9" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -1290,14 +1304,14 @@
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="4" x14ac:dyDescent="0" defaultColWidth="9" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -1560,14 +1574,14 @@
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="4" x14ac:dyDescent="0" defaultColWidth="9" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -1830,14 +1844,14 @@
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="4" x14ac:dyDescent="0" defaultColWidth="9" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -2100,14 +2114,14 @@
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="4" x14ac:dyDescent="0" defaultColWidth="9" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -2116,13 +2130,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2370,6 +2384,6 @@
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>